<commit_message>
Rename sewer density feature
</commit_message>
<xml_diff>
--- a/data/hannam_sinkhole_data.xlsx
+++ b/data/hannam_sinkhole_data.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="training_data" sheetId="1" r:id="R93208ca64d9a4d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="training_data" sheetId="1" r:id="R80d89356c37443d0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -326,6 +326,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
@@ -380,7 +383,7 @@
         <x:v>sewer_Y_20</x:v>
       </x:c>
       <x:c r="R1" t="str">
-        <x:v>sewer_total_density_km_km2</x:v>
+        <x:v>sewer_Density</x:v>
       </x:c>
       <x:c r="S1" t="str">
         <x:v>cavity_count</x:v>

</xml_diff>